<commit_message>
Update with 0.05, 0.10 and 0.15
</commit_message>
<xml_diff>
--- a/outputs_batch_contour_bias/manual_channel_TRUE_contour_overlap/manual_channel_TRUE_contour_overlap_summary.xlsx
+++ b/outputs_batch_contour_bias/manual_channel_TRUE_contour_overlap/manual_channel_TRUE_contour_overlap_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,50 +446,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>n_images</t>
+          <t>mean_contour_preference_ratio</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>mean_contour_preference_ratio</t>
+          <t>sem_contour_preference_ratio</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>sem_contour_preference_ratio</t>
+          <t>mean_activation_on_contour_pct</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>mean_activation_on_contour_pct</t>
+          <t>sem_activation_on_contour_pct</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>sem_activation_on_contour_pct</t>
+          <t>mean_contour_area_pct</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>mean_contour_area_pct</t>
+          <t>mean_contour_enrichment</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>mean_contour_enrichment</t>
+          <t>sem_contour_enrichment</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>sem_contour_enrichment</t>
+          <t>mean_dice_top_activation</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>mean_dice_top_activation</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>sem_dice_top_activation</t>
         </is>
@@ -507,37 +502,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>128</v>
+        <v>3200</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>1.779860973358154</v>
       </c>
       <c r="E2" t="n">
-        <v>1.779860973358154</v>
+        <v>0.0215885229408741</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1065115034580231</v>
+        <v>2.867997407913208</v>
       </c>
       <c r="G2" t="n">
-        <v>2.867997407913208</v>
+        <v>0.03304437920451164</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1633336544036865</v>
+        <v>1.6533203125</v>
       </c>
       <c r="I2" t="n">
-        <v>1.6533203125</v>
+        <v>1.734689520220136</v>
       </c>
       <c r="J2" t="n">
-        <v>1.734689520220136</v>
+        <v>0.01998667641829434</v>
       </c>
       <c r="K2" t="n">
-        <v>0.09879129857041831</v>
+        <v>0.1077050583601519</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1077050583601519</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.007185890072556277</v>
+        <v>0.001445195627785251</v>
       </c>
     </row>
     <row r="3">
@@ -552,37 +544,34 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>128</v>
+        <v>3200</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>1.6089186668396</v>
       </c>
       <c r="E3" t="n">
-        <v>1.60891854763031</v>
+        <v>0.02186270989477634</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1084671840071678</v>
+        <v>2.594673871994019</v>
       </c>
       <c r="G3" t="n">
-        <v>2.594673871994019</v>
+        <v>0.03396747633814812</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1686663627624512</v>
+        <v>1.6533203125</v>
       </c>
       <c r="I3" t="n">
-        <v>1.6533203125</v>
+        <v>1.569371560395293</v>
       </c>
       <c r="J3" t="n">
-        <v>1.569371560395293</v>
+        <v>0.02054500540860659</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1020167437686084</v>
+        <v>0.09431217451092003</v>
       </c>
       <c r="L3" t="n">
-        <v>0.09431217451092004</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.00788391824656552</v>
+        <v>0.001585432198986434</v>
       </c>
     </row>
     <row r="4">
@@ -597,37 +586,34 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>128</v>
+        <v>3200</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>1.638879299163818</v>
       </c>
       <c r="E4" t="n">
-        <v>1.638879179954529</v>
+        <v>0.01980802044272423</v>
       </c>
       <c r="F4" t="n">
-        <v>0.09080178290605545</v>
+        <v>1.34024703502655</v>
       </c>
       <c r="G4" t="n">
-        <v>1.34024703502655</v>
+        <v>0.01577582396566868</v>
       </c>
       <c r="H4" t="n">
-        <v>0.07260064780712128</v>
+        <v>0.8271484375000001</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8271484375000001</v>
+        <v>1.620322202641874</v>
       </c>
       <c r="J4" t="n">
-        <v>1.620322202641874</v>
+        <v>0.01907254160320127</v>
       </c>
       <c r="K4" t="n">
-        <v>0.087772209422582</v>
+        <v>0.05273117064391707</v>
       </c>
       <c r="L4" t="n">
-        <v>0.05273117064391707</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.003868768200915446</v>
+        <v>0.0008200187466197811</v>
       </c>
     </row>
     <row r="5">
@@ -642,37 +628,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>128</v>
+        <v>3200</v>
       </c>
       <c r="D5" t="n">
-        <v>25</v>
+        <v>1.516645193099976</v>
       </c>
       <c r="E5" t="n">
-        <v>1.516645193099976</v>
+        <v>0.02090194262564182</v>
       </c>
       <c r="F5" t="n">
-        <v>0.09876125305891037</v>
+        <v>1.239927291870117</v>
       </c>
       <c r="G5" t="n">
-        <v>1.239927291870117</v>
+        <v>0.01675325073301792</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07932960987091064</v>
+        <v>0.8271484375000001</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8271484375000001</v>
+        <v>1.499038449962639</v>
       </c>
       <c r="J5" t="n">
-        <v>1.499038449962639</v>
+        <v>0.02025422520028388</v>
       </c>
       <c r="K5" t="n">
-        <v>0.09590734873600877</v>
+        <v>0.04778017860441168</v>
       </c>
       <c r="L5" t="n">
-        <v>0.04778017860441169</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.004324722560594723</v>
+        <v>0.0009053059007303512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>